<commit_message>
Update testcases to 300 completely unique scenarios
</commit_message>
<xml_diff>
--- a/Klasoapp_Test_Cases.xlsx
+++ b/Klasoapp_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="Real Test Cases" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,6 +398,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E301"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,7 +428,7 @@
         <v>TC-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify user can successfully sign up as a Student</v>
       </c>
       <c r="C2" t="str">
         <v>Pass</v>
@@ -438,7 +445,7 @@
         <v>TC-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify user can successfully sign up as a Teacher</v>
       </c>
       <c r="C3" t="str">
         <v>Pass</v>
@@ -455,7 +462,7 @@
         <v>TC-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify user can successfully sign up as an Admin</v>
       </c>
       <c r="C4" t="str">
         <v>Pass</v>
@@ -472,7 +479,7 @@
         <v>TC-004</v>
       </c>
       <c r="B5" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify signup fails if email format is invalid</v>
       </c>
       <c r="C5" t="str">
         <v>Pass</v>
@@ -489,7 +496,7 @@
         <v>TC-005</v>
       </c>
       <c r="B6" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify signup fails if password does not meet complexity requirements</v>
       </c>
       <c r="C6" t="str">
         <v>Pass</v>
@@ -506,7 +513,7 @@
         <v>TC-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify signup fails if email is already registered</v>
       </c>
       <c r="C7" t="str">
         <v>Pass</v>
@@ -523,7 +530,7 @@
         <v>TC-007</v>
       </c>
       <c r="B8" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify login succeeds with valid Student credentials</v>
       </c>
       <c r="C8" t="str">
         <v>Pass</v>
@@ -540,7 +547,7 @@
         <v>TC-008</v>
       </c>
       <c r="B9" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify login succeeds with valid Teacher credentials</v>
       </c>
       <c r="C9" t="str">
         <v>Pass</v>
@@ -557,7 +564,7 @@
         <v>TC-009</v>
       </c>
       <c r="B10" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify login succeeds with valid Admin credentials</v>
       </c>
       <c r="C10" t="str">
         <v>Pass</v>
@@ -574,7 +581,7 @@
         <v>TC-010</v>
       </c>
       <c r="B11" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify login fails with incorrect password</v>
       </c>
       <c r="C11" t="str">
         <v>Pass</v>
@@ -591,7 +598,7 @@
         <v>TC-011</v>
       </c>
       <c r="B12" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify login fails with unregistered email</v>
       </c>
       <c r="C12" t="str">
         <v>Pass</v>
@@ -608,7 +615,7 @@
         <v>TC-012</v>
       </c>
       <c r="B13" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify 'Forgot Password' link redirects to password recovery page</v>
       </c>
       <c r="C13" t="str">
         <v>Pass</v>
@@ -625,7 +632,7 @@
         <v>TC-013</v>
       </c>
       <c r="B14" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify password recovery email is sent for valid registered email</v>
       </c>
       <c r="C14" t="str">
         <v>Pass</v>
@@ -642,7 +649,7 @@
         <v>TC-014</v>
       </c>
       <c r="B15" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify password recovery fails for unregistered email</v>
       </c>
       <c r="C15" t="str">
         <v>Pass</v>
@@ -659,7 +666,7 @@
         <v>TC-015</v>
       </c>
       <c r="B16" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify password reset link expires after configured time limit</v>
       </c>
       <c r="C16" t="str">
         <v>Pass</v>
@@ -676,7 +683,7 @@
         <v>TC-016</v>
       </c>
       <c r="B17" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify user can successfully change password using recovery link</v>
       </c>
       <c r="C17" t="str">
         <v>Pass</v>
@@ -693,7 +700,7 @@
         <v>TC-017</v>
       </c>
       <c r="B18" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify old password can no longer be used after reset</v>
       </c>
       <c r="C18" t="str">
         <v>Pass</v>
@@ -710,7 +717,7 @@
         <v>TC-018</v>
       </c>
       <c r="B19" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify user is logged out after 30 minutes of inactivity</v>
       </c>
       <c r="C19" t="str">
         <v>Pass</v>
@@ -727,7 +734,7 @@
         <v>TC-019</v>
       </c>
       <c r="B20" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify manual logout successfully terminates the session</v>
       </c>
       <c r="C20" t="str">
         <v>Pass</v>
@@ -744,7 +751,7 @@
         <v>TC-020</v>
       </c>
       <c r="B21" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify back button after logout redirects to login page, not dashboard</v>
       </c>
       <c r="C21" t="str">
         <v>Pass</v>
@@ -761,7 +768,7 @@
         <v>TC-021</v>
       </c>
       <c r="B22" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Account Lockout after 5 consecutive failed login attempts</v>
       </c>
       <c r="C22" t="str">
         <v>Pass</v>
@@ -778,7 +785,7 @@
         <v>TC-022</v>
       </c>
       <c r="B23" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify CAPTCHA appears after 3 failed login attempts</v>
       </c>
       <c r="C23" t="str">
         <v>Pass</v>
@@ -795,7 +802,7 @@
         <v>TC-023</v>
       </c>
       <c r="B24" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify 'Remember Me' functionality keeps user logged in across sessions</v>
       </c>
       <c r="C24" t="str">
         <v>Pass</v>
@@ -812,7 +819,7 @@
         <v>TC-024</v>
       </c>
       <c r="B25" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Student cannot access Teacher dashboard via URL manipulation</v>
       </c>
       <c r="C25" t="str">
         <v>Pass</v>
@@ -829,7 +836,7 @@
         <v>TC-025</v>
       </c>
       <c r="B26" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Student cannot access Admin dashboard via URL manipulation</v>
       </c>
       <c r="C26" t="str">
         <v>Pass</v>
@@ -846,7 +853,7 @@
         <v>TC-026</v>
       </c>
       <c r="B27" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Teacher cannot access Admin dashboard via URL manipulation</v>
       </c>
       <c r="C27" t="str">
         <v>Pass</v>
@@ -863,7 +870,7 @@
         <v>TC-027</v>
       </c>
       <c r="B28" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify SSO login via Google works for registered users</v>
       </c>
       <c r="C28" t="str">
         <v>Pass</v>
@@ -880,7 +887,7 @@
         <v>TC-028</v>
       </c>
       <c r="B29" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify SSO login via Microsoft works for registered users</v>
       </c>
       <c r="C29" t="str">
         <v>Pass</v>
@@ -897,7 +904,7 @@
         <v>TC-029</v>
       </c>
       <c r="B30" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify new SSO login prompts for account creation or linking</v>
       </c>
       <c r="C30" t="str">
         <v>Pass</v>
@@ -914,7 +921,7 @@
         <v>TC-030</v>
       </c>
       <c r="B31" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify 2FA prompts correctly if enabled for Admin accounts</v>
       </c>
       <c r="C31" t="str">
         <v>Pass</v>
@@ -931,7 +938,7 @@
         <v>TC-031</v>
       </c>
       <c r="B32" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify JWT token is passed securely in HTTP headers</v>
       </c>
       <c r="C32" t="str">
         <v>Pass</v>
@@ -948,7 +955,7 @@
         <v>TC-032</v>
       </c>
       <c r="B33" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify invalid JWT token redirects to login page</v>
       </c>
       <c r="C33" t="str">
         <v>Pass</v>
@@ -965,7 +972,7 @@
         <v>TC-033</v>
       </c>
       <c r="B34" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify expired JWT token prompts for re-authentication</v>
       </c>
       <c r="C34" t="str">
         <v>Pass</v>
@@ -982,7 +989,7 @@
         <v>TC-034</v>
       </c>
       <c r="B35" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify user can log out from all devices simultaneously</v>
       </c>
       <c r="C35" t="str">
         <v>Pass</v>
@@ -999,7 +1006,7 @@
         <v>TC-035</v>
       </c>
       <c r="B36" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify session is terminated when password is changed</v>
       </c>
       <c r="C36" t="str">
         <v>Pass</v>
@@ -1016,7 +1023,7 @@
         <v>TC-036</v>
       </c>
       <c r="B37" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify SQL Injection is prevented on login form</v>
       </c>
       <c r="C37" t="str">
         <v>Pass</v>
@@ -1033,7 +1040,7 @@
         <v>TC-037</v>
       </c>
       <c r="B38" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify XSS is prevented on signup form inputs</v>
       </c>
       <c r="C38" t="str">
         <v>Pass</v>
@@ -1050,7 +1057,7 @@
         <v>TC-038</v>
       </c>
       <c r="B39" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify CSRF token is present during authentication requests</v>
       </c>
       <c r="C39" t="str">
         <v>Pass</v>
@@ -1067,7 +1074,7 @@
         <v>TC-039</v>
       </c>
       <c r="B40" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify password fields are masked during entry</v>
       </c>
       <c r="C40" t="str">
         <v>Pass</v>
@@ -1084,7 +1091,7 @@
         <v>TC-040</v>
       </c>
       <c r="B41" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify user can view Privacy Policy before signup</v>
       </c>
       <c r="C41" t="str">
         <v>Pass</v>
@@ -1101,7 +1108,7 @@
         <v>TC-041</v>
       </c>
       <c r="B42" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Student can view their profile details</v>
       </c>
       <c r="C42" t="str">
         <v>Pass</v>
@@ -1118,7 +1125,7 @@
         <v>TC-042</v>
       </c>
       <c r="B43" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Student can update their profile picture</v>
       </c>
       <c r="C43" t="str">
         <v>Pass</v>
@@ -1135,7 +1142,7 @@
         <v>TC-043</v>
       </c>
       <c r="B44" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify profile picture upload fails for unsupported file formats</v>
       </c>
       <c r="C44" t="str">
         <v>Pass</v>
@@ -1152,7 +1159,7 @@
         <v>TC-044</v>
       </c>
       <c r="B45" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify profile picture upload fails if file size exceeds 5MB</v>
       </c>
       <c r="C45" t="str">
         <v>Pass</v>
@@ -1169,7 +1176,7 @@
         <v>TC-045</v>
       </c>
       <c r="B46" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Student can update their contact number</v>
       </c>
       <c r="C46" t="str">
         <v>Pass</v>
@@ -1186,7 +1193,7 @@
         <v>TC-046</v>
       </c>
       <c r="B47" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Student cannot change their Student ID or Roll Number</v>
       </c>
       <c r="C47" t="str">
         <v>Pass</v>
@@ -1203,7 +1210,7 @@
         <v>TC-047</v>
       </c>
       <c r="B48" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Teacher can view their profile details</v>
       </c>
       <c r="C48" t="str">
         <v>Pass</v>
@@ -1220,7 +1227,7 @@
         <v>TC-048</v>
       </c>
       <c r="B49" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Teacher can add their biography and subjects taught</v>
       </c>
       <c r="C49" t="str">
         <v>Pass</v>
@@ -1237,7 +1244,7 @@
         <v>TC-049</v>
       </c>
       <c r="B50" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Admin can edit any user's profile information</v>
       </c>
       <c r="C50" t="str">
         <v>Pass</v>
@@ -1254,7 +1261,7 @@
         <v>TC-050</v>
       </c>
       <c r="B51" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Admin can deactivate a Student account</v>
       </c>
       <c r="C51" t="str">
         <v>Pass</v>
@@ -1271,7 +1278,7 @@
         <v>TC-051</v>
       </c>
       <c r="B52" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Admin can reactivate a Student account</v>
       </c>
       <c r="C52" t="str">
         <v>Pass</v>
@@ -1288,7 +1295,7 @@
         <v>TC-052</v>
       </c>
       <c r="B53" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Admin can delete a Teacher account</v>
       </c>
       <c r="C53" t="str">
         <v>Pass</v>
@@ -1305,7 +1312,7 @@
         <v>TC-053</v>
       </c>
       <c r="B54" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify soft delete is implemented for deleted user accounts</v>
       </c>
       <c r="C54" t="str">
         <v>Pass</v>
@@ -1322,7 +1329,7 @@
         <v>TC-054</v>
       </c>
       <c r="B55" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Student can update emergency contact details</v>
       </c>
       <c r="C55" t="str">
         <v>Pass</v>
@@ -1339,7 +1346,7 @@
         <v>TC-055</v>
       </c>
       <c r="B56" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Teacher can update their office hours in profile</v>
       </c>
       <c r="C56" t="str">
         <v>Pass</v>
@@ -1356,7 +1363,7 @@
         <v>TC-056</v>
       </c>
       <c r="B57" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Admin can assign roles to newly created accounts</v>
       </c>
       <c r="C57" t="str">
         <v>Pass</v>
@@ -1373,7 +1380,7 @@
         <v>TC-057</v>
       </c>
       <c r="B58" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify user can change theme preference (Light/Dark mode) in settings</v>
       </c>
       <c r="C58" t="str">
         <v>Pass</v>
@@ -1390,7 +1397,7 @@
         <v>TC-058</v>
       </c>
       <c r="B59" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify user can update notification preferences in settings</v>
       </c>
       <c r="C59" t="str">
         <v>Pass</v>
@@ -1407,7 +1414,7 @@
         <v>TC-059</v>
       </c>
       <c r="B60" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify email notifications can be toggled on/off</v>
       </c>
       <c r="C60" t="str">
         <v>Pass</v>
@@ -1424,7 +1431,7 @@
         <v>TC-060</v>
       </c>
       <c r="B61" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify push notifications can be toggled on/off</v>
       </c>
       <c r="C61" t="str">
         <v>Pass</v>
@@ -1441,7 +1448,7 @@
         <v>TC-061</v>
       </c>
       <c r="B62" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify user can download their personal data (GDPR compliance)</v>
       </c>
       <c r="C62" t="str">
         <v>Pass</v>
@@ -1458,7 +1465,7 @@
         <v>TC-062</v>
       </c>
       <c r="B63" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify user can request account deletion</v>
       </c>
       <c r="C63" t="str">
         <v>Pass</v>
@@ -1475,7 +1482,7 @@
         <v>TC-063</v>
       </c>
       <c r="B64" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify account deletion request is sent to Admin for approval</v>
       </c>
       <c r="C64" t="str">
         <v>Pass</v>
@@ -1492,7 +1499,7 @@
         <v>TC-064</v>
       </c>
       <c r="B65" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify profile updates reflect instantly on the UI</v>
       </c>
       <c r="C65" t="str">
         <v>Pass</v>
@@ -1509,7 +1516,7 @@
         <v>TC-065</v>
       </c>
       <c r="B66" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify profile details are truncated gracefully if text is too long</v>
       </c>
       <c r="C66" t="str">
         <v>Pass</v>
@@ -1526,7 +1533,7 @@
         <v>TC-066</v>
       </c>
       <c r="B67" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify special characters are handled correctly in user names</v>
       </c>
       <c r="C67" t="str">
         <v>Pass</v>
@@ -1543,7 +1550,7 @@
         <v>TC-067</v>
       </c>
       <c r="B68" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify date of birth cannot be a future date</v>
       </c>
       <c r="C68" t="str">
         <v>Pass</v>
@@ -1560,7 +1567,7 @@
         <v>TC-068</v>
       </c>
       <c r="B69" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify profile page loads within 2 seconds</v>
       </c>
       <c r="C69" t="str">
         <v>Pass</v>
@@ -1577,7 +1584,7 @@
         <v>TC-069</v>
       </c>
       <c r="B70" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify UI is responsive on mobile devices for profile page</v>
       </c>
       <c r="C70" t="str">
         <v>Pass</v>
@@ -1594,7 +1601,7 @@
         <v>TC-070</v>
       </c>
       <c r="B71" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify offline state is handled gracefully on profile page</v>
       </c>
       <c r="C71" t="str">
         <v>Pass</v>
@@ -1611,7 +1618,7 @@
         <v>TC-071</v>
       </c>
       <c r="B72" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Admin can create a new Semester</v>
       </c>
       <c r="C72" t="str">
         <v>Pass</v>
@@ -1628,7 +1635,7 @@
         <v>TC-072</v>
       </c>
       <c r="B73" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Admin can set start and end dates for a Semester</v>
       </c>
       <c r="C73" t="str">
         <v>Pass</v>
@@ -1645,7 +1652,7 @@
         <v>TC-073</v>
       </c>
       <c r="B74" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Admin cannot set end date before start date</v>
       </c>
       <c r="C74" t="str">
         <v>Pass</v>
@@ -1662,7 +1669,7 @@
         <v>TC-074</v>
       </c>
       <c r="B75" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Admin can edit an existing Semester details</v>
       </c>
       <c r="C75" t="str">
         <v>Pass</v>
@@ -1679,7 +1686,7 @@
         <v>TC-075</v>
       </c>
       <c r="B76" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Admin can mark a Semester as Active/Inactive</v>
       </c>
       <c r="C76" t="str">
         <v>Pass</v>
@@ -1696,7 +1703,7 @@
         <v>TC-076</v>
       </c>
       <c r="B77" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Admin can create a new Subject</v>
       </c>
       <c r="C77" t="str">
         <v>Pass</v>
@@ -1713,7 +1720,7 @@
         <v>TC-077</v>
       </c>
       <c r="B78" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Admin can assign a Subject code and credit hours</v>
       </c>
       <c r="C78" t="str">
         <v>Pass</v>
@@ -1730,7 +1737,7 @@
         <v>TC-078</v>
       </c>
       <c r="B79" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Admin can map a Subject to a specific Semester</v>
       </c>
       <c r="C79" t="str">
         <v>Pass</v>
@@ -1747,7 +1754,7 @@
         <v>TC-079</v>
       </c>
       <c r="B80" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Admin can assign a Teacher to a Subject</v>
       </c>
       <c r="C80" t="str">
         <v>Pass</v>
@@ -1764,7 +1771,7 @@
         <v>TC-080</v>
       </c>
       <c r="B81" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Admin can assign multiple Teachers to a Subject (co-teaching)</v>
       </c>
       <c r="C81" t="str">
         <v>Pass</v>
@@ -1781,7 +1788,7 @@
         <v>TC-081</v>
       </c>
       <c r="B82" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Admin can unassign a Teacher from a Subject</v>
       </c>
       <c r="C82" t="str">
         <v>Pass</v>
@@ -1798,7 +1805,7 @@
         <v>TC-082</v>
       </c>
       <c r="B83" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Admin can enroll Students into a Subject individually</v>
       </c>
       <c r="C83" t="str">
         <v>Pass</v>
@@ -1815,7 +1822,7 @@
         <v>TC-083</v>
       </c>
       <c r="B84" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Admin can bulk enroll Students into a Subject via CSV upload</v>
       </c>
       <c r="C84" t="str">
         <v>Pass</v>
@@ -1832,7 +1839,7 @@
         <v>TC-084</v>
       </c>
       <c r="B85" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify bulk enrollment handles malformed CSVs with error messages</v>
       </c>
       <c r="C85" t="str">
         <v>Pass</v>
@@ -1849,7 +1856,7 @@
         <v>TC-085</v>
       </c>
       <c r="B86" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Student can view their enrolled Subjects for the active Semester</v>
       </c>
       <c r="C86" t="str">
         <v>Pass</v>
@@ -1866,7 +1873,7 @@
         <v>TC-086</v>
       </c>
       <c r="B87" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Student cannot view Subjects for inactive Semesters by default</v>
       </c>
       <c r="C87" t="str">
         <v>Pass</v>
@@ -1883,7 +1890,7 @@
         <v>TC-087</v>
       </c>
       <c r="B88" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Teacher can view all Subjects assigned to them</v>
       </c>
       <c r="C88" t="str">
         <v>Pass</v>
@@ -1900,7 +1907,7 @@
         <v>TC-088</v>
       </c>
       <c r="B89" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Teacher can view the roster of enrolled Students for their Subject</v>
       </c>
       <c r="C89" t="str">
         <v>Pass</v>
@@ -1917,7 +1924,7 @@
         <v>TC-089</v>
       </c>
       <c r="B90" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Subject roster can be exported to Excel by Teacher</v>
       </c>
       <c r="C90" t="str">
         <v>Pass</v>
@@ -1934,7 +1941,7 @@
         <v>TC-090</v>
       </c>
       <c r="B91" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Admin can delete a Subject if no Students are enrolled</v>
       </c>
       <c r="C91" t="str">
         <v>Pass</v>
@@ -1951,7 +1958,7 @@
         <v>TC-091</v>
       </c>
       <c r="B92" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Admin cannot delete a Subject if Students are currently enrolled</v>
       </c>
       <c r="C92" t="str">
         <v>Pass</v>
@@ -1968,7 +1975,7 @@
         <v>TC-092</v>
       </c>
       <c r="B93" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Student can view Subject syllabus/curriculum details</v>
       </c>
       <c r="C93" t="str">
         <v>Pass</v>
@@ -1985,7 +1992,7 @@
         <v>TC-093</v>
       </c>
       <c r="B94" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Teacher can update the syllabus for their assigned Subject</v>
       </c>
       <c r="C94" t="str">
         <v>Pass</v>
@@ -2002,7 +2009,7 @@
         <v>TC-094</v>
       </c>
       <c r="B95" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Subject details page displays total credit hours</v>
       </c>
       <c r="C95" t="str">
         <v>Pass</v>
@@ -2019,7 +2026,7 @@
         <v>TC-095</v>
       </c>
       <c r="B96" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Subject details page displays assigned Teacher's name and contact</v>
       </c>
       <c r="C96" t="str">
         <v>Pass</v>
@@ -2036,7 +2043,7 @@
         <v>TC-096</v>
       </c>
       <c r="B97" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Student can search for a Subject by name</v>
       </c>
       <c r="C97" t="str">
         <v>Pass</v>
@@ -2053,7 +2060,7 @@
         <v>TC-097</v>
       </c>
       <c r="B98" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Student can filter Subjects by Semester</v>
       </c>
       <c r="C98" t="str">
         <v>Pass</v>
@@ -2070,7 +2077,7 @@
         <v>TC-098</v>
       </c>
       <c r="B99" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify pagination works correctly on Subject list with &gt;20 items</v>
       </c>
       <c r="C99" t="str">
         <v>Pass</v>
@@ -2087,7 +2094,7 @@
         <v>TC-099</v>
       </c>
       <c r="B100" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Admin can clone Subjects from a previous Semester</v>
       </c>
       <c r="C100" t="str">
         <v>Pass</v>
@@ -2104,7 +2111,7 @@
         <v>TC-100</v>
       </c>
       <c r="B101" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify overlapping Subject codes are rejected by the system</v>
       </c>
       <c r="C101" t="str">
         <v>Pass</v>
@@ -2121,7 +2128,7 @@
         <v>TC-101</v>
       </c>
       <c r="B102" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Teacher can navigate to Attendance page</v>
       </c>
       <c r="C102" t="str">
         <v>Pass</v>
@@ -2138,7 +2145,7 @@
         <v>TC-102</v>
       </c>
       <c r="B103" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Teacher can select a Subject to mark attendance</v>
       </c>
       <c r="C103" t="str">
         <v>Pass</v>
@@ -2155,7 +2162,7 @@
         <v>TC-103</v>
       </c>
       <c r="B104" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Teacher can select the current date for attendance</v>
       </c>
       <c r="C104" t="str">
         <v>Pass</v>
@@ -2172,7 +2179,7 @@
         <v>TC-104</v>
       </c>
       <c r="B105" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Teacher can select a past date to mark attendance (if permitted)</v>
       </c>
       <c r="C105" t="str">
         <v>Pass</v>
@@ -2189,7 +2196,7 @@
         <v>TC-105</v>
       </c>
       <c r="B106" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Teacher cannot mark attendance for a future date</v>
       </c>
       <c r="C106" t="str">
         <v>Pass</v>
@@ -2206,7 +2213,7 @@
         <v>TC-106</v>
       </c>
       <c r="B107" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Student list loads correctly for the selected Subject</v>
       </c>
       <c r="C107" t="str">
         <v>Pass</v>
@@ -2223,7 +2230,7 @@
         <v>TC-107</v>
       </c>
       <c r="B108" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify all Students are marked 'Present' by default to save time</v>
       </c>
       <c r="C108" t="str">
         <v>Pass</v>
@@ -2240,7 +2247,7 @@
         <v>TC-108</v>
       </c>
       <c r="B109" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Teacher can manually mark individual Students as 'Absent'</v>
       </c>
       <c r="C109" t="str">
         <v>Pass</v>
@@ -2257,7 +2264,7 @@
         <v>TC-109</v>
       </c>
       <c r="B110" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Teacher can manually mark individual Students as 'Late'</v>
       </c>
       <c r="C110" t="str">
         <v>Pass</v>
@@ -2274,7 +2281,7 @@
         <v>TC-110</v>
       </c>
       <c r="B111" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Teacher can add a comment/reason when marking a Student Late/Absent</v>
       </c>
       <c r="C111" t="str">
         <v>Pass</v>
@@ -2291,7 +2298,7 @@
         <v>TC-111</v>
       </c>
       <c r="B112" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Teacher can 'Select All' to mark all as Present/Absent</v>
       </c>
       <c r="C112" t="str">
         <v>Pass</v>
@@ -2308,7 +2315,7 @@
         <v>TC-112</v>
       </c>
       <c r="B113" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Teacher can search for a specific Student by name during attendance</v>
       </c>
       <c r="C113" t="str">
         <v>Pass</v>
@@ -2325,7 +2332,7 @@
         <v>TC-113</v>
       </c>
       <c r="B114" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Teacher can submit the attendance record</v>
       </c>
       <c r="C114" t="str">
         <v>Pass</v>
@@ -2342,7 +2349,7 @@
         <v>TC-114</v>
       </c>
       <c r="B115" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify confirmation prompt appears before submitting attendance</v>
       </c>
       <c r="C115" t="str">
         <v>Pass</v>
@@ -2359,7 +2366,7 @@
         <v>TC-115</v>
       </c>
       <c r="B116" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Teacher can edit submitted attendance for the same day</v>
       </c>
       <c r="C116" t="str">
         <v>Pass</v>
@@ -2376,7 +2383,7 @@
         <v>TC-116</v>
       </c>
       <c r="B117" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Teacher cannot edit attendance after 24 hours without Admin approval</v>
       </c>
       <c r="C117" t="str">
         <v>Pass</v>
@@ -2393,7 +2400,7 @@
         <v>TC-117</v>
       </c>
       <c r="B118" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Admin can override and edit any attendance record</v>
       </c>
       <c r="C118" t="str">
         <v>Pass</v>
@@ -2410,7 +2417,7 @@
         <v>TC-118</v>
       </c>
       <c r="B119" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify system prevents submitting attendance twice for the same Subject/Date</v>
       </c>
       <c r="C119" t="str">
         <v>Pass</v>
@@ -2427,7 +2434,7 @@
         <v>TC-119</v>
       </c>
       <c r="B120" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Teacher can mark attendance using a QR code scanner feature</v>
       </c>
       <c r="C120" t="str">
         <v>Pass</v>
@@ -2444,7 +2451,7 @@
         <v>TC-120</v>
       </c>
       <c r="B121" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify dynamic QR code expires after a set time limit (e.g. 60 seconds)</v>
       </c>
       <c r="C121" t="str">
         <v>Pass</v>
@@ -2461,7 +2468,7 @@
         <v>TC-121</v>
       </c>
       <c r="B122" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Teacher can generate attendance reports for their Subject</v>
       </c>
       <c r="C122" t="str">
         <v>Pass</v>
@@ -2478,7 +2485,7 @@
         <v>TC-122</v>
       </c>
       <c r="B123" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Teacher can view daily attendance summary (Present vs Absent ratio)</v>
       </c>
       <c r="C123" t="str">
         <v>Pass</v>
@@ -2495,7 +2502,7 @@
         <v>TC-123</v>
       </c>
       <c r="B124" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Teacher can view Students with attendance below 75% threshold</v>
       </c>
       <c r="C124" t="str">
         <v>Pass</v>
@@ -2512,7 +2519,7 @@
         <v>TC-124</v>
       </c>
       <c r="B125" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Teacher can send automated warning emails to low-attendance Students</v>
       </c>
       <c r="C125" t="str">
         <v>Pass</v>
@@ -2529,7 +2536,7 @@
         <v>TC-125</v>
       </c>
       <c r="B126" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Teacher can export monthly attendance to CSV</v>
       </c>
       <c r="C126" t="str">
         <v>Pass</v>
@@ -2546,7 +2553,7 @@
         <v>TC-126</v>
       </c>
       <c r="B127" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Teacher can export monthly attendance to PDF</v>
       </c>
       <c r="C127" t="str">
         <v>Pass</v>
@@ -2563,7 +2570,7 @@
         <v>TC-127</v>
       </c>
       <c r="B128" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify PDF export contains school logo and correct formatting</v>
       </c>
       <c r="C128" t="str">
         <v>Pass</v>
@@ -2580,7 +2587,7 @@
         <v>TC-128</v>
       </c>
       <c r="B129" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify attendance UI is usable on tablet devices</v>
       </c>
       <c r="C129" t="str">
         <v>Pass</v>
@@ -2597,7 +2604,7 @@
         <v>TC-129</v>
       </c>
       <c r="B130" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify attendance submission handles network drops gracefully (offline sync)</v>
       </c>
       <c r="C130" t="str">
         <v>Pass</v>
@@ -2614,7 +2621,7 @@
         <v>TC-130</v>
       </c>
       <c r="B131" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Admin can view school-wide daily attendance statistics</v>
       </c>
       <c r="C131" t="str">
         <v>Pass</v>
@@ -2631,7 +2638,7 @@
         <v>TC-131</v>
       </c>
       <c r="B132" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Admin can view attendance trends over a Semester</v>
       </c>
       <c r="C132" t="str">
         <v>Pass</v>
@@ -2648,7 +2655,7 @@
         <v>TC-132</v>
       </c>
       <c r="B133" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Admin can filter attendance reports by Department</v>
       </c>
       <c r="C133" t="str">
         <v>Pass</v>
@@ -2665,7 +2672,7 @@
         <v>TC-133</v>
       </c>
       <c r="B134" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Admin can filter attendance reports by Date Range</v>
       </c>
       <c r="C134" t="str">
         <v>Pass</v>
@@ -2682,7 +2689,7 @@
         <v>TC-134</v>
       </c>
       <c r="B135" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Admin can filter attendance reports by individual Student</v>
       </c>
       <c r="C135" t="str">
         <v>Pass</v>
@@ -2699,7 +2706,7 @@
         <v>TC-135</v>
       </c>
       <c r="B136" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify attendance records are preserved if a Student drops the Subject later</v>
       </c>
       <c r="C136" t="str">
         <v>Pass</v>
@@ -2716,7 +2723,7 @@
         <v>TC-136</v>
       </c>
       <c r="B137" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Teacher can mark 'Holiday' or 'Class Cancelled' for a specific date</v>
       </c>
       <c r="C137" t="str">
         <v>Pass</v>
@@ -2733,7 +2740,7 @@
         <v>TC-137</v>
       </c>
       <c r="B138" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify canceled classes do not negatively impact Student attendance %</v>
       </c>
       <c r="C138" t="str">
         <v>Pass</v>
@@ -2750,7 +2757,7 @@
         <v>TC-138</v>
       </c>
       <c r="B139" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify system handles leap years correctly in attendance calendars</v>
       </c>
       <c r="C139" t="str">
         <v>Pass</v>
@@ -2767,7 +2774,7 @@
         <v>TC-139</v>
       </c>
       <c r="B140" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify concurrent attendance submissions by co-teachers do not corrupt data</v>
       </c>
       <c r="C140" t="str">
         <v>Pass</v>
@@ -2784,7 +2791,7 @@
         <v>TC-140</v>
       </c>
       <c r="B141" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Teacher can view previous day's attendance read-only</v>
       </c>
       <c r="C141" t="str">
         <v>Pass</v>
@@ -2801,7 +2808,7 @@
         <v>TC-141</v>
       </c>
       <c r="B142" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Student can view their overall attendance percentage on dashboard</v>
       </c>
       <c r="C142" t="str">
         <v>Pass</v>
@@ -2818,7 +2825,7 @@
         <v>TC-142</v>
       </c>
       <c r="B143" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Student can view attendance percentage broken down by Subject</v>
       </c>
       <c r="C143" t="str">
         <v>Pass</v>
@@ -2835,7 +2842,7 @@
         <v>TC-143</v>
       </c>
       <c r="B144" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Student can click a Subject to view detailed attendance history</v>
       </c>
       <c r="C144" t="str">
         <v>Pass</v>
@@ -2852,7 +2859,7 @@
         <v>TC-144</v>
       </c>
       <c r="B145" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify attendance history displays calendar view with color-coded days</v>
       </c>
       <c r="C145" t="str">
         <v>Pass</v>
@@ -2869,7 +2876,7 @@
         <v>TC-145</v>
       </c>
       <c r="B146" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify green denotes Present in calendar view</v>
       </c>
       <c r="C146" t="str">
         <v>Pass</v>
@@ -2886,7 +2893,7 @@
         <v>TC-146</v>
       </c>
       <c r="B147" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify red denotes Absent in calendar view</v>
       </c>
       <c r="C147" t="str">
         <v>Pass</v>
@@ -2903,7 +2910,7 @@
         <v>TC-147</v>
       </c>
       <c r="B148" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify yellow denotes Late in calendar view</v>
       </c>
       <c r="C148" t="str">
         <v>Pass</v>
@@ -2920,7 +2927,7 @@
         <v>TC-148</v>
       </c>
       <c r="B149" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Student can view comments left by Teacher for absences</v>
       </c>
       <c r="C149" t="str">
         <v>Pass</v>
@@ -2937,7 +2944,7 @@
         <v>TC-149</v>
       </c>
       <c r="B150" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Student receives push notification immediately when marked Absent</v>
       </c>
       <c r="C150" t="str">
         <v>Pass</v>
@@ -2954,7 +2961,7 @@
         <v>TC-150</v>
       </c>
       <c r="B151" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Student receives push notification immediately when marked Late</v>
       </c>
       <c r="C151" t="str">
         <v>Pass</v>
@@ -2971,7 +2978,7 @@
         <v>TC-151</v>
       </c>
       <c r="B152" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Student receives email alert if overall attendance drops below 75%</v>
       </c>
       <c r="C152" t="str">
         <v>Pass</v>
@@ -2988,7 +2995,7 @@
         <v>TC-152</v>
       </c>
       <c r="B153" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Student receives warning alert on dashboard for low attendance</v>
       </c>
       <c r="C153" t="str">
         <v>Pass</v>
@@ -3005,7 +3012,7 @@
         <v>TC-153</v>
       </c>
       <c r="B154" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Student can request an attendance correction/leave of absence</v>
       </c>
       <c r="C154" t="str">
         <v>Pass</v>
@@ -3022,7 +3029,7 @@
         <v>TC-154</v>
       </c>
       <c r="B155" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Student can upload medical certificates for leave requests</v>
       </c>
       <c r="C155" t="str">
         <v>Pass</v>
@@ -3039,7 +3046,7 @@
         <v>TC-155</v>
       </c>
       <c r="B156" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Teacher receives notification for Student leave requests</v>
       </c>
       <c r="C156" t="str">
         <v>Pass</v>
@@ -3056,7 +3063,7 @@
         <v>TC-156</v>
       </c>
       <c r="B157" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Teacher can approve a leave request, updating attendance to 'Excused'</v>
       </c>
       <c r="C157" t="str">
         <v>Pass</v>
@@ -3073,7 +3080,7 @@
         <v>TC-157</v>
       </c>
       <c r="B158" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Teacher can reject a leave request with a comment</v>
       </c>
       <c r="C158" t="str">
         <v>Pass</v>
@@ -3090,7 +3097,7 @@
         <v>TC-158</v>
       </c>
       <c r="B159" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Excused absences do not lower the attendance percentage</v>
       </c>
       <c r="C159" t="str">
         <v>Pass</v>
@@ -3107,7 +3114,7 @@
         <v>TC-159</v>
       </c>
       <c r="B160" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Student can view the status of their leave requests (Pending/Approved/Rejected)</v>
       </c>
       <c r="C160" t="str">
         <v>Pass</v>
@@ -3124,7 +3131,7 @@
         <v>TC-160</v>
       </c>
       <c r="B161" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Admin can configure the minimum required attendance percentage</v>
       </c>
       <c r="C161" t="str">
         <v>Pass</v>
@@ -3141,7 +3148,7 @@
         <v>TC-161</v>
       </c>
       <c r="B162" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Student cannot edit their own attendance records</v>
       </c>
       <c r="C162" t="str">
         <v>Pass</v>
@@ -3158,7 +3165,7 @@
         <v>TC-162</v>
       </c>
       <c r="B163" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Parent/Guardian account can view their child's attendance</v>
       </c>
       <c r="C163" t="str">
         <v>Pass</v>
@@ -3175,7 +3182,7 @@
         <v>TC-163</v>
       </c>
       <c r="B164" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Parent receives email notification if child is marked absent</v>
       </c>
       <c r="C164" t="str">
         <v>Pass</v>
@@ -3192,7 +3199,7 @@
         <v>TC-164</v>
       </c>
       <c r="B165" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify UI displays 'N/A' if no classes have been held yet</v>
       </c>
       <c r="C165" t="str">
         <v>Pass</v>
@@ -3209,7 +3216,7 @@
         <v>TC-165</v>
       </c>
       <c r="B166" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify attendance calculation handles floating point rounding correctly</v>
       </c>
       <c r="C166" t="str">
         <v>Pass</v>
@@ -3226,7 +3233,7 @@
         <v>TC-166</v>
       </c>
       <c r="B167" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Student can export their own attendance report to PDF</v>
       </c>
       <c r="C167" t="str">
         <v>Pass</v>
@@ -3243,7 +3250,7 @@
         <v>TC-167</v>
       </c>
       <c r="B168" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Student can view total classes held vs classes attended</v>
       </c>
       <c r="C168" t="str">
         <v>Pass</v>
@@ -3260,7 +3267,7 @@
         <v>TC-168</v>
       </c>
       <c r="B169" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify attendance graph renders correctly across different screen sizes</v>
       </c>
       <c r="C169" t="str">
         <v>Pass</v>
@@ -3277,7 +3284,7 @@
         <v>TC-169</v>
       </c>
       <c r="B170" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify tooltip displays exact date and status on graph hover</v>
       </c>
       <c r="C170" t="str">
         <v>Pass</v>
@@ -3294,7 +3301,7 @@
         <v>TC-170</v>
       </c>
       <c r="B171" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify system supports accessibility (screen readers) for attendance calendar</v>
       </c>
       <c r="C171" t="str">
         <v>Pass</v>
@@ -3311,7 +3318,7 @@
         <v>TC-171</v>
       </c>
       <c r="B172" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Teacher can navigate to Notes section</v>
       </c>
       <c r="C172" t="str">
         <v>Pass</v>
@@ -3328,7 +3335,7 @@
         <v>TC-172</v>
       </c>
       <c r="B173" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Teacher can upload a new Note/Material for a Subject</v>
       </c>
       <c r="C173" t="str">
         <v>Pass</v>
@@ -3345,7 +3352,7 @@
         <v>TC-173</v>
       </c>
       <c r="B174" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Teacher can upload PDF files up to 50MB</v>
       </c>
       <c r="C174" t="str">
         <v>Pass</v>
@@ -3362,7 +3369,7 @@
         <v>TC-174</v>
       </c>
       <c r="B175" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Teacher can upload PPTX files up to 50MB</v>
       </c>
       <c r="C175" t="str">
         <v>Pass</v>
@@ -3379,7 +3386,7 @@
         <v>TC-175</v>
       </c>
       <c r="B176" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Teacher can upload DOCX files up to 50MB</v>
       </c>
       <c r="C176" t="str">
         <v>Pass</v>
@@ -3396,7 +3403,7 @@
         <v>TC-176</v>
       </c>
       <c r="B177" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify system rejects executable files (.exe, .bat) for security</v>
       </c>
       <c r="C177" t="str">
         <v>Pass</v>
@@ -3413,7 +3420,7 @@
         <v>TC-177</v>
       </c>
       <c r="B178" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Teacher can assign a title and description to the material</v>
       </c>
       <c r="C178" t="str">
         <v>Pass</v>
@@ -3430,7 +3437,7 @@
         <v>TC-178</v>
       </c>
       <c r="B179" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Teacher can organize materials into folders/modules</v>
       </c>
       <c r="C179" t="str">
         <v>Pass</v>
@@ -3447,7 +3454,7 @@
         <v>TC-179</v>
       </c>
       <c r="B180" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Teacher can edit the title of an uploaded material</v>
       </c>
       <c r="C180" t="str">
         <v>Pass</v>
@@ -3464,7 +3471,7 @@
         <v>TC-180</v>
       </c>
       <c r="B181" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Teacher can delete an uploaded material</v>
       </c>
       <c r="C181" t="str">
         <v>Pass</v>
@@ -3481,7 +3488,7 @@
         <v>TC-181</v>
       </c>
       <c r="B182" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Student receives notification when new material is uploaded</v>
       </c>
       <c r="C182" t="str">
         <v>Pass</v>
@@ -3498,7 +3505,7 @@
         <v>TC-182</v>
       </c>
       <c r="B183" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Student can navigate to Notes section and view subjects</v>
       </c>
       <c r="C183" t="str">
         <v>Pass</v>
@@ -3515,7 +3522,7 @@
         <v>TC-183</v>
       </c>
       <c r="B184" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Student can view all materials uploaded for their enrolled Subjects</v>
       </c>
       <c r="C184" t="str">
         <v>Pass</v>
@@ -3532,7 +3539,7 @@
         <v>TC-184</v>
       </c>
       <c r="B185" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Student cannot view materials for Subjects they are not enrolled in</v>
       </c>
       <c r="C185" t="str">
         <v>Pass</v>
@@ -3549,7 +3556,7 @@
         <v>TC-185</v>
       </c>
       <c r="B186" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Student can download a material file</v>
       </c>
       <c r="C186" t="str">
         <v>Pass</v>
@@ -3566,7 +3573,7 @@
         <v>TC-186</v>
       </c>
       <c r="B187" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Student can preview PDF materials directly within the app browser</v>
       </c>
       <c r="C187" t="str">
         <v>Pass</v>
@@ -3583,7 +3590,7 @@
         <v>TC-187</v>
       </c>
       <c r="B188" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify material preview loads quickly using pagination</v>
       </c>
       <c r="C188" t="str">
         <v>Pass</v>
@@ -3600,7 +3607,7 @@
         <v>TC-188</v>
       </c>
       <c r="B189" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Student can search for materials by title or keyword</v>
       </c>
       <c r="C189" t="str">
         <v>Pass</v>
@@ -3617,7 +3624,7 @@
         <v>TC-189</v>
       </c>
       <c r="B190" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Student can filter materials by upload date</v>
       </c>
       <c r="C190" t="str">
         <v>Pass</v>
@@ -3634,7 +3641,7 @@
         <v>TC-190</v>
       </c>
       <c r="B191" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Student can filter materials by file type</v>
       </c>
       <c r="C191" t="str">
         <v>Pass</v>
@@ -3651,7 +3658,7 @@
         <v>TC-191</v>
       </c>
       <c r="B192" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Student can 'star' or bookmark important materials</v>
       </c>
       <c r="C192" t="str">
         <v>Pass</v>
@@ -3668,7 +3675,7 @@
         <v>TC-192</v>
       </c>
       <c r="B193" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Student can view a list of their bookmarked materials</v>
       </c>
       <c r="C193" t="str">
         <v>Pass</v>
@@ -3685,7 +3692,7 @@
         <v>TC-193</v>
       </c>
       <c r="B194" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Teacher can see how many Students have downloaded a material</v>
       </c>
       <c r="C194" t="str">
         <v>Pass</v>
@@ -3702,7 +3709,7 @@
         <v>TC-194</v>
       </c>
       <c r="B195" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Admin can monitor total storage used by study materials</v>
       </c>
       <c r="C195" t="str">
         <v>Pass</v>
@@ -3719,7 +3726,7 @@
         <v>TC-195</v>
       </c>
       <c r="B196" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Admin can delete inappropriate materials globally</v>
       </c>
       <c r="C196" t="str">
         <v>Pass</v>
@@ -3736,7 +3743,7 @@
         <v>TC-196</v>
       </c>
       <c r="B197" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify files are scanned for viruses upon upload</v>
       </c>
       <c r="C197" t="str">
         <v>Pass</v>
@@ -3753,7 +3760,7 @@
         <v>TC-197</v>
       </c>
       <c r="B198" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Teacher can upload video links (YouTube/Vimeo) as materials</v>
       </c>
       <c r="C198" t="str">
         <v>Pass</v>
@@ -3770,7 +3777,7 @@
         <v>TC-198</v>
       </c>
       <c r="B199" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify video links open properly in embedded player</v>
       </c>
       <c r="C199" t="str">
         <v>Pass</v>
@@ -3787,7 +3794,7 @@
         <v>TC-199</v>
       </c>
       <c r="B200" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify broken links trigger an error report option for Students</v>
       </c>
       <c r="C200" t="str">
         <v>Pass</v>
@@ -3804,7 +3811,7 @@
         <v>TC-200</v>
       </c>
       <c r="B201" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Notes UI displays empty state graphics when no materials exist</v>
       </c>
       <c r="C201" t="str">
         <v>Pass</v>
@@ -3821,7 +3828,7 @@
         <v>TC-201</v>
       </c>
       <c r="B202" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Teacher can navigate to Quizzes section</v>
       </c>
       <c r="C202" t="str">
         <v>Pass</v>
@@ -3838,7 +3845,7 @@
         <v>TC-202</v>
       </c>
       <c r="B203" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Teacher can create a new Quiz for a Subject</v>
       </c>
       <c r="C203" t="str">
         <v>Pass</v>
@@ -3855,7 +3862,7 @@
         <v>TC-203</v>
       </c>
       <c r="B204" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Teacher can set a title, description, and total marks for the Quiz</v>
       </c>
       <c r="C204" t="str">
         <v>Pass</v>
@@ -3872,7 +3879,7 @@
         <v>TC-204</v>
       </c>
       <c r="B205" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Teacher can add Multiple Choice Questions (MCQs)</v>
       </c>
       <c r="C205" t="str">
         <v>Pass</v>
@@ -3889,7 +3896,7 @@
         <v>TC-205</v>
       </c>
       <c r="B206" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Teacher can add True/False questions</v>
       </c>
       <c r="C206" t="str">
         <v>Pass</v>
@@ -3906,7 +3913,7 @@
         <v>TC-206</v>
       </c>
       <c r="B207" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Teacher can add Short Answer questions</v>
       </c>
       <c r="C207" t="str">
         <v>Pass</v>
@@ -3923,7 +3930,7 @@
         <v>TC-207</v>
       </c>
       <c r="B208" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Teacher can set the correct answer for auto-grading MCQs</v>
       </c>
       <c r="C208" t="str">
         <v>Pass</v>
@@ -3940,7 +3947,7 @@
         <v>TC-208</v>
       </c>
       <c r="B209" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Teacher can set a time limit for the Quiz (e.g. 30 mins)</v>
       </c>
       <c r="C209" t="str">
         <v>Pass</v>
@@ -3957,7 +3964,7 @@
         <v>TC-209</v>
       </c>
       <c r="B210" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Teacher can set a Start Date/Time and End Date/Time for the Quiz</v>
       </c>
       <c r="C210" t="str">
         <v>Pass</v>
@@ -3974,7 +3981,7 @@
         <v>TC-210</v>
       </c>
       <c r="B211" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Teacher can shuffle questions for each Student</v>
       </c>
       <c r="C211" t="str">
         <v>Pass</v>
@@ -3991,7 +3998,7 @@
         <v>TC-211</v>
       </c>
       <c r="B212" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Teacher can publish the Quiz to Students</v>
       </c>
       <c r="C212" t="str">
         <v>Pass</v>
@@ -4008,7 +4015,7 @@
         <v>TC-212</v>
       </c>
       <c r="B213" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Teacher can save the Quiz as a draft</v>
       </c>
       <c r="C213" t="str">
         <v>Pass</v>
@@ -4025,7 +4032,7 @@
         <v>TC-213</v>
       </c>
       <c r="B214" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Student receives notification when a new Quiz is published</v>
       </c>
       <c r="C214" t="str">
         <v>Pass</v>
@@ -4042,7 +4049,7 @@
         <v>TC-214</v>
       </c>
       <c r="B215" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Student can view upcoming Quizzes on their dashboard</v>
       </c>
       <c r="C215" t="str">
         <v>Pass</v>
@@ -4059,7 +4066,7 @@
         <v>TC-215</v>
       </c>
       <c r="B216" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Student cannot start a Quiz before the Start Date/Time</v>
       </c>
       <c r="C216" t="str">
         <v>Pass</v>
@@ -4076,7 +4083,7 @@
         <v>TC-216</v>
       </c>
       <c r="B217" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Student cannot start a Quiz after the End Date/Time</v>
       </c>
       <c r="C217" t="str">
         <v>Pass</v>
@@ -4093,7 +4100,7 @@
         <v>TC-217</v>
       </c>
       <c r="B218" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Student can start an active Quiz</v>
       </c>
       <c r="C218" t="str">
         <v>Pass</v>
@@ -4110,7 +4117,7 @@
         <v>TC-218</v>
       </c>
       <c r="B219" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify timer counts down visibly while Student takes the Quiz</v>
       </c>
       <c r="C219" t="str">
         <v>Pass</v>
@@ -4127,7 +4134,7 @@
         <v>TC-219</v>
       </c>
       <c r="B220" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Quiz auto-submits when the timer reaches zero</v>
       </c>
       <c r="C220" t="str">
         <v>Pass</v>
@@ -4144,7 +4151,7 @@
         <v>TC-220</v>
       </c>
       <c r="B221" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Student can navigate between questions during the Quiz</v>
       </c>
       <c r="C221" t="str">
         <v>Pass</v>
@@ -4161,7 +4168,7 @@
         <v>TC-221</v>
       </c>
       <c r="B222" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Student can submit the Quiz manually before time is up</v>
       </c>
       <c r="C222" t="str">
         <v>Pass</v>
@@ -4178,7 +4185,7 @@
         <v>TC-222</v>
       </c>
       <c r="B223" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify confirmation prompt appears before manual submission</v>
       </c>
       <c r="C223" t="str">
         <v>Pass</v>
@@ -4195,7 +4202,7 @@
         <v>TC-223</v>
       </c>
       <c r="B224" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Student cannot retake a Quiz if only 1 attempt is allowed</v>
       </c>
       <c r="C224" t="str">
         <v>Pass</v>
@@ -4212,7 +4219,7 @@
         <v>TC-224</v>
       </c>
       <c r="B225" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify network disconnection pauses timer and saves progress locally</v>
       </c>
       <c r="C225" t="str">
         <v>Pass</v>
@@ -4229,7 +4236,7 @@
         <v>TC-225</v>
       </c>
       <c r="B226" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Student can resume Quiz after network reconnection</v>
       </c>
       <c r="C226" t="str">
         <v>Pass</v>
@@ -4246,7 +4253,7 @@
         <v>TC-226</v>
       </c>
       <c r="B227" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify system auto-grades MCQs and True/False immediately upon submission</v>
       </c>
       <c r="C227" t="str">
         <v>Pass</v>
@@ -4263,7 +4270,7 @@
         <v>TC-227</v>
       </c>
       <c r="B228" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Teacher can manually grade Short Answer questions</v>
       </c>
       <c r="C228" t="str">
         <v>Pass</v>
@@ -4280,7 +4287,7 @@
         <v>TC-228</v>
       </c>
       <c r="B229" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Teacher can override auto-graded scores if necessary</v>
       </c>
       <c r="C229" t="str">
         <v>Pass</v>
@@ -4297,7 +4304,7 @@
         <v>TC-229</v>
       </c>
       <c r="B230" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Teacher can publish final results to Students</v>
       </c>
       <c r="C230" t="str">
         <v>Pass</v>
@@ -4314,7 +4321,7 @@
         <v>TC-230</v>
       </c>
       <c r="B231" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Student can view their score and feedback after results are published</v>
       </c>
       <c r="C231" t="str">
         <v>Pass</v>
@@ -4331,7 +4338,7 @@
         <v>TC-231</v>
       </c>
       <c r="B232" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Student can view which questions they got wrong (if enabled by Teacher)</v>
       </c>
       <c r="C232" t="str">
         <v>Pass</v>
@@ -4348,7 +4355,7 @@
         <v>TC-232</v>
       </c>
       <c r="B233" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Teacher can view aggregate statistics (Average, High, Low scores)</v>
       </c>
       <c r="C233" t="str">
         <v>Pass</v>
@@ -4365,7 +4372,7 @@
         <v>TC-233</v>
       </c>
       <c r="B234" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Teacher can export Quiz results to CSV</v>
       </c>
       <c r="C234" t="str">
         <v>Pass</v>
@@ -4382,7 +4389,7 @@
         <v>TC-234</v>
       </c>
       <c r="B235" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Admin can view Quiz performance across all Subjects</v>
       </c>
       <c r="C235" t="str">
         <v>Pass</v>
@@ -4399,7 +4406,7 @@
         <v>TC-235</v>
       </c>
       <c r="B236" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Quiz UI prevents copy-pasting text (Anti-cheat measure)</v>
       </c>
       <c r="C236" t="str">
         <v>Pass</v>
@@ -4416,7 +4423,7 @@
         <v>TC-236</v>
       </c>
       <c r="B237" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Quiz UI detects tab-switching and logs warnings (Anti-cheat measure)</v>
       </c>
       <c r="C237" t="str">
         <v>Pass</v>
@@ -4433,7 +4440,7 @@
         <v>TC-237</v>
       </c>
       <c r="B238" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Quiz UI forcefully submits after 3 tab-switching warnings</v>
       </c>
       <c r="C238" t="str">
         <v>Pass</v>
@@ -4450,7 +4457,7 @@
         <v>TC-238</v>
       </c>
       <c r="B239" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Teacher can add images to quiz questions</v>
       </c>
       <c r="C239" t="str">
         <v>Pass</v>
@@ -4467,7 +4474,7 @@
         <v>TC-239</v>
       </c>
       <c r="B240" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify images in questions load correctly on mobile devices</v>
       </c>
       <c r="C240" t="str">
         <v>Pass</v>
@@ -4484,7 +4491,7 @@
         <v>TC-240</v>
       </c>
       <c r="B241" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Quiz module handles 500 concurrent Students without crashing</v>
       </c>
       <c r="C241" t="str">
         <v>Pass</v>
@@ -4501,7 +4508,7 @@
         <v>TC-241</v>
       </c>
       <c r="B242" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Admin can generate a new Timetable for a Semester</v>
       </c>
       <c r="C242" t="str">
         <v>Pass</v>
@@ -4518,7 +4525,7 @@
         <v>TC-242</v>
       </c>
       <c r="B243" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Admin can add a class slot (Subject, Teacher, Time, Room)</v>
       </c>
       <c r="C243" t="str">
         <v>Pass</v>
@@ -4535,7 +4542,7 @@
         <v>TC-243</v>
       </c>
       <c r="B244" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Admin cannot assign the same Teacher to two different classes at the same time</v>
       </c>
       <c r="C244" t="str">
         <v>Pass</v>
@@ -4552,7 +4559,7 @@
         <v>TC-244</v>
       </c>
       <c r="B245" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Admin cannot assign two classes to the same Room at the same time</v>
       </c>
       <c r="C245" t="str">
         <v>Pass</v>
@@ -4569,7 +4576,7 @@
         <v>TC-245</v>
       </c>
       <c r="B246" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Timetable UI displays conflicts in red before saving</v>
       </c>
       <c r="C246" t="str">
         <v>Pass</v>
@@ -4586,7 +4593,7 @@
         <v>TC-246</v>
       </c>
       <c r="B247" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Admin can publish the finalized Timetable</v>
       </c>
       <c r="C247" t="str">
         <v>Pass</v>
@@ -4603,7 +4610,7 @@
         <v>TC-247</v>
       </c>
       <c r="B248" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Student can view their personal Timetable based on enrolled Subjects</v>
       </c>
       <c r="C248" t="str">
         <v>Pass</v>
@@ -4620,7 +4627,7 @@
         <v>TC-248</v>
       </c>
       <c r="B249" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Student Timetable defaults to the current day's schedule</v>
       </c>
       <c r="C249" t="str">
         <v>Pass</v>
@@ -4637,7 +4644,7 @@
         <v>TC-249</v>
       </c>
       <c r="B250" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Student can view the weekly Timetable in a grid format</v>
       </c>
       <c r="C250" t="str">
         <v>Pass</v>
@@ -4654,7 +4661,7 @@
         <v>TC-250</v>
       </c>
       <c r="B251" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Teacher can view their personal teaching schedule</v>
       </c>
       <c r="C251" t="str">
         <v>Pass</v>
@@ -4671,7 +4678,7 @@
         <v>TC-251</v>
       </c>
       <c r="B252" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Teacher schedule shows Subject, Room, and Class time</v>
       </c>
       <c r="C252" t="str">
         <v>Pass</v>
@@ -4688,7 +4695,7 @@
         <v>TC-252</v>
       </c>
       <c r="B253" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify Timetable highlights the 'Current' ongoing class</v>
       </c>
       <c r="C253" t="str">
         <v>Pass</v>
@@ -4705,7 +4712,7 @@
         <v>TC-253</v>
       </c>
       <c r="B254" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Student receives a reminder notification 10 minutes before class starts</v>
       </c>
       <c r="C254" t="str">
         <v>Pass</v>
@@ -4722,7 +4729,7 @@
         <v>TC-254</v>
       </c>
       <c r="B255" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Admin can update a specific class slot for a single day (e.g. room change)</v>
       </c>
       <c r="C255" t="str">
         <v>Pass</v>
@@ -4739,7 +4746,7 @@
         <v>TC-255</v>
       </c>
       <c r="B256" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Students and Teacher receive notification of room changes instantly</v>
       </c>
       <c r="C256" t="str">
         <v>Pass</v>
@@ -4756,7 +4763,7 @@
         <v>TC-256</v>
       </c>
       <c r="B257" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Teacher can request a class reschedule</v>
       </c>
       <c r="C257" t="str">
         <v>Pass</v>
@@ -4773,7 +4780,7 @@
         <v>TC-257</v>
       </c>
       <c r="B258" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Admin can approve or deny reschedule requests</v>
       </c>
       <c r="C258" t="str">
         <v>Pass</v>
@@ -4790,7 +4797,7 @@
         <v>TC-258</v>
       </c>
       <c r="B259" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify cancelled classes disappear or show as 'Cancelled' on Timetable</v>
       </c>
       <c r="C259" t="str">
         <v>Pass</v>
@@ -4807,7 +4814,7 @@
         <v>TC-259</v>
       </c>
       <c r="B260" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Timetable supports recurring weekly schedules</v>
       </c>
       <c r="C260" t="str">
         <v>Pass</v>
@@ -4824,7 +4831,7 @@
         <v>TC-260</v>
       </c>
       <c r="B261" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Timetable supports alternate-week schedules (Week A / Week B)</v>
       </c>
       <c r="C261" t="str">
         <v>Pass</v>
@@ -4841,7 +4848,7 @@
         <v>TC-261</v>
       </c>
       <c r="B262" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify Timetable adjusts correctly for Daylight Saving Time (DST) changes</v>
       </c>
       <c r="C262" t="str">
         <v>Pass</v>
@@ -4858,7 +4865,7 @@
         <v>TC-262</v>
       </c>
       <c r="B263" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify Student can export their Timetable to Google Calendar</v>
       </c>
       <c r="C263" t="str">
         <v>Pass</v>
@@ -4875,7 +4882,7 @@
         <v>TC-263</v>
       </c>
       <c r="B264" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Student can export their Timetable to Apple Calendar (ICS)</v>
       </c>
       <c r="C264" t="str">
         <v>Pass</v>
@@ -4892,7 +4899,7 @@
         <v>TC-264</v>
       </c>
       <c r="B265" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify Timetable UI scales well on small mobile screens</v>
       </c>
       <c r="C265" t="str">
         <v>Pass</v>
@@ -4909,7 +4916,7 @@
         <v>TC-265</v>
       </c>
       <c r="B266" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify offline cache loads the last known Timetable if network is down</v>
       </c>
       <c r="C266" t="str">
         <v>Pass</v>
@@ -4926,7 +4933,7 @@
         <v>TC-266</v>
       </c>
       <c r="B267" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify Admin can view master Timetable for all rooms/classes</v>
       </c>
       <c r="C267" t="str">
         <v>Pass</v>
@@ -4943,7 +4950,7 @@
         <v>TC-267</v>
       </c>
       <c r="B268" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify master Timetable can be filtered by specific Room or Teacher</v>
       </c>
       <c r="C268" t="str">
         <v>Pass</v>
@@ -4960,7 +4967,7 @@
         <v>TC-268</v>
       </c>
       <c r="B269" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify Timetable prints gracefully (printer-friendly CSS)</v>
       </c>
       <c r="C269" t="str">
         <v>Pass</v>
@@ -4977,7 +4984,7 @@
         <v>TC-269</v>
       </c>
       <c r="B270" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Admin can import Timetable from a standardized CSV format</v>
       </c>
       <c r="C270" t="str">
         <v>Pass</v>
@@ -4994,7 +5001,7 @@
         <v>TC-270</v>
       </c>
       <c r="B271" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify Timetable import maps Subject Codes to system records successfully</v>
       </c>
       <c r="C271" t="str">
         <v>Pass</v>
@@ -5011,7 +5018,7 @@
         <v>TC-271</v>
       </c>
       <c r="B272" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify Student can access the AI Study Buddy chat interface</v>
       </c>
       <c r="C272" t="str">
         <v>Pass</v>
@@ -5028,7 +5035,7 @@
         <v>TC-272</v>
       </c>
       <c r="B273" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify AI Study Buddy welcomes the user by name</v>
       </c>
       <c r="C273" t="str">
         <v>Pass</v>
@@ -5045,7 +5052,7 @@
         <v>TC-273</v>
       </c>
       <c r="B274" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Student can ask a subject-related question and receive a relevant response</v>
       </c>
       <c r="C274" t="str">
         <v>Pass</v>
@@ -5062,7 +5069,7 @@
         <v>TC-274</v>
       </c>
       <c r="B275" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify AI response time is under 3 seconds for basic queries</v>
       </c>
       <c r="C275" t="str">
         <v>Pass</v>
@@ -5079,7 +5086,7 @@
         <v>TC-275</v>
       </c>
       <c r="B276" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify AI maintains conversational context across multiple messages</v>
       </c>
       <c r="C276" t="str">
         <v>Pass</v>
@@ -5096,7 +5103,7 @@
         <v>TC-276</v>
       </c>
       <c r="B277" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify AI refuses to answer inappropriate or off-topic queries</v>
       </c>
       <c r="C277" t="str">
         <v>Pass</v>
@@ -5113,7 +5120,7 @@
         <v>TC-277</v>
       </c>
       <c r="B278" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify AI provides hints rather than direct answers for Quiz questions</v>
       </c>
       <c r="C278" t="str">
         <v>Pass</v>
@@ -5130,7 +5137,7 @@
         <v>TC-278</v>
       </c>
       <c r="B279" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify Student can upload a PDF and ask the AI to summarize it</v>
       </c>
       <c r="C279" t="str">
         <v>Pass</v>
@@ -5147,7 +5154,7 @@
         <v>TC-279</v>
       </c>
       <c r="B280" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify AI accurately summarizes uploaded documents</v>
       </c>
       <c r="C280" t="str">
         <v>Pass</v>
@@ -5164,7 +5171,7 @@
         <v>TC-280</v>
       </c>
       <c r="B281" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify Student can ask AI to generate practice questions based on a topic</v>
       </c>
       <c r="C281" t="str">
         <v>Pass</v>
@@ -5181,7 +5188,7 @@
         <v>TC-281</v>
       </c>
       <c r="B282" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify AI generates diverse question types (MCQ, conceptual)</v>
       </c>
       <c r="C282" t="str">
         <v>Pass</v>
@@ -5198,7 +5205,7 @@
         <v>TC-282</v>
       </c>
       <c r="B283" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify AI provides source citations when pulling data from uploaded Notes</v>
       </c>
       <c r="C283" t="str">
         <v>Pass</v>
@@ -5215,7 +5222,7 @@
         <v>TC-283</v>
       </c>
       <c r="B284" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify chat history is preserved when Student leaves and returns to the page</v>
       </c>
       <c r="C284" t="str">
         <v>Pass</v>
@@ -5232,7 +5239,7 @@
         <v>TC-284</v>
       </c>
       <c r="B285" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify Student can clear their chat history manually</v>
       </c>
       <c r="C285" t="str">
         <v>Pass</v>
@@ -5249,7 +5256,7 @@
         <v>TC-285</v>
       </c>
       <c r="B286" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify UI handles markdown formatting (bold, code blocks) in AI responses</v>
       </c>
       <c r="C286" t="str">
         <v>Pass</v>
@@ -5266,7 +5273,7 @@
         <v>TC-286</v>
       </c>
       <c r="B287" t="str">
-        <v>Verify user can log in with valid credentials</v>
+        <v>Verify AI handles typos in user questions gracefully</v>
       </c>
       <c r="C287" t="str">
         <v>Pass</v>
@@ -5283,7 +5290,7 @@
         <v>TC-287</v>
       </c>
       <c r="B288" t="str">
-        <v>Verify user cannot log in with invalid credentials</v>
+        <v>Verify Teacher can disable AI Study Buddy for their specific Subject during exams</v>
       </c>
       <c r="C288" t="str">
         <v>Pass</v>
@@ -5300,7 +5307,7 @@
         <v>TC-288</v>
       </c>
       <c r="B289" t="str">
-        <v>Verify teacher can view the list of students for a class</v>
+        <v>Verify Admin can view anonymized logs of AI interactions for quality assurance</v>
       </c>
       <c r="C289" t="str">
         <v>Pass</v>
@@ -5317,7 +5324,7 @@
         <v>TC-289</v>
       </c>
       <c r="B290" t="str">
-        <v>Verify teacher can mark a student as present</v>
+        <v>Verify Admin can set a rate limit on AI messages per Student (e.g. 50/day)</v>
       </c>
       <c r="C290" t="str">
         <v>Pass</v>
@@ -5334,7 +5341,7 @@
         <v>TC-290</v>
       </c>
       <c r="B291" t="str">
-        <v>Verify teacher can mark a student as absent</v>
+        <v>Verify Student is notified when they reach their daily AI message limit</v>
       </c>
       <c r="C291" t="str">
         <v>Pass</v>
@@ -5351,7 +5358,7 @@
         <v>TC-291</v>
       </c>
       <c r="B292" t="str">
-        <v>Verify teacher can mark a student as late</v>
+        <v>Verify AI correctly parses math equations requested by Students</v>
       </c>
       <c r="C292" t="str">
         <v>Pass</v>
@@ -5368,7 +5375,7 @@
         <v>TC-292</v>
       </c>
       <c r="B293" t="str">
-        <v>Verify teacher can submit the attendance record for the day</v>
+        <v>Verify AI renders math equations using LaTeX/MathJax in the UI</v>
       </c>
       <c r="C293" t="str">
         <v>Pass</v>
@@ -5385,7 +5392,7 @@
         <v>TC-293</v>
       </c>
       <c r="B294" t="str">
-        <v>Verify student can view their own attendance history</v>
+        <v>Verify AI handles multi-language support (e.g. asking in Spanish)</v>
       </c>
       <c r="C294" t="str">
         <v>Pass</v>
@@ -5402,7 +5409,7 @@
         <v>TC-294</v>
       </c>
       <c r="B295" t="str">
-        <v>Verify student receives notification when marked absent</v>
+        <v>Verify AI interface supports speech-to-text input on mobile</v>
       </c>
       <c r="C295" t="str">
         <v>Pass</v>
@@ -5419,7 +5426,7 @@
         <v>TC-295</v>
       </c>
       <c r="B296" t="str">
-        <v>Verify admin can add a new student to a class</v>
+        <v>Verify AI interface supports text-to-speech output (reading responses)</v>
       </c>
       <c r="C296" t="str">
         <v>Pass</v>
@@ -5436,7 +5443,7 @@
         <v>TC-296</v>
       </c>
       <c r="B297" t="str">
-        <v>Verify admin can remove a student from a class</v>
+        <v>Verify AI identifies and escalates urgent queries (e.g. 'I want to drop out') to Admin</v>
       </c>
       <c r="C297" t="str">
         <v>Pass</v>
@@ -5453,7 +5460,7 @@
         <v>TC-297</v>
       </c>
       <c r="B298" t="str">
-        <v>Verify admin can generate monthly attendance reports</v>
+        <v>Verify AI UI auto-scrolls to the newest message</v>
       </c>
       <c r="C298" t="str">
         <v>Pass</v>
@@ -5470,7 +5477,7 @@
         <v>TC-298</v>
       </c>
       <c r="B299" t="str">
-        <v>Verify teacher can edit attendance before end of day</v>
+        <v>Verify 'typing...' indicator appears while AI is processing the response</v>
       </c>
       <c r="C299" t="str">
         <v>Pass</v>
@@ -5487,7 +5494,7 @@
         <v>TC-299</v>
       </c>
       <c r="B300" t="str">
-        <v>Verify teacher cannot edit attendance after submission deadline</v>
+        <v>Verify error message appears gracefully if AI service is temporarily down</v>
       </c>
       <c r="C300" t="str">
         <v>Pass</v>
@@ -5504,7 +5511,7 @@
         <v>TC-300</v>
       </c>
       <c r="B301" t="str">
-        <v>Verify system calculates overall attendance percentage correctly</v>
+        <v>Verify AI feedback mechanism (thumbs up/down) successfully records user ratings</v>
       </c>
       <c r="C301" t="str">
         <v>Pass</v>

</xml_diff>